<commit_message>
feat(m7): improve allocation rules for sprint 3
</commit_message>
<xml_diff>
--- a/test-evidence/M7-Chai-Zihan/UT-M7-table.xlsx
+++ b/test-evidence/M7-Chai-Zihan/UT-M7-table.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="39">
   <si>
     <t>Test Name/ID</t>
   </si>
@@ -95,10 +95,55 @@
     <t>Sprint 3</t>
   </si>
   <si>
-    <t/>
+    <t>Project has maxStudents = 2 and another application is still pending</t>
+  </si>
+  <si>
+    <t>Teacher accepts one pending application for this project</t>
+  </si>
+  <si>
+    <t>The selected application becomes accepted; the other pending application remains pending; topic status remains requested</t>
+  </si>
+  <si>
+    <t>System does not auto reject other pending applications before the project is full</t>
+  </si>
+  <si>
+    <t>Other pending application remained pending and topic status stayed requested</t>
   </si>
   <si>
     <t>UT-M7-S3-02</t>
+  </si>
+  <si>
+    <t>Project reaches maxStudents after approval and still has other pending applications</t>
+  </si>
+  <si>
+    <t>Teacher accepts a pending application that fills the project capacity</t>
+  </si>
+  <si>
+    <t>The selected application becomes accepted; other pending applications are auto rejected; topic status becomes agreed; conflict log is saved</t>
+  </si>
+  <si>
+    <t>System auto rejects remaining pending applications only when the project is full</t>
+  </si>
+  <si>
+    <t>Other pending applications were rejected, topic became agreed, and conflict log was saved</t>
+  </si>
+  <si>
+    <t>UT-M7-S3-03</t>
+  </si>
+  <si>
+    <t>Student already has an accepted application or project has reached capacity</t>
+  </si>
+  <si>
+    <t>Teacher tries to accept another conflicting application</t>
+  </si>
+  <si>
+    <t>System rejects the approval and saves a conflict log</t>
+  </si>
+  <si>
+    <t>System records allocation conflict when student or project capacity conflict occurs</t>
+  </si>
+  <si>
+    <t>Conflict log was saved and approval was rejected</t>
   </si>
 </sst>
 </file>
@@ -129,7 +174,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -294,13 +338,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.05"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.05"/>
+        <fgColor theme="0" tint="-0.15"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.15"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -645,19 +689,19 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -666,7 +710,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -795,19 +839,21 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1154,12 +1200,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H5"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="4" outlineLevelCol="7"/>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="5" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
     <col min="2" max="2" width="9" customWidth="1"/>
-    <col min="3" max="3" width="35.3636363636364" customWidth="1"/>
+    <col min="3" max="3" width="83.6363636363636" customWidth="1"/>
     <col min="4" max="4" width="73.6363636363636" customWidth="1"/>
     <col min="5" max="5" width="70.2727272727273" customWidth="1"/>
     <col min="6" max="6" width="30.9090909090909" customWidth="1"/>
@@ -1226,7 +1272,7 @@
       <c r="B3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="4" t="s">
         <v>16</v>
       </c>
       <c r="D3" s="5" t="s">
@@ -1246,53 +1292,81 @@
       </c>
     </row>
     <row r="4" ht="42" customHeight="1" spans="1:8">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" s="6"/>
-      <c r="H4" s="4" t="s">
-        <v>22</v>
+      <c r="D4" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1" spans="1:8">
-      <c r="A5" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" s="4" t="s">
+      <c r="A5" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>22</v>
+      <c r="C5" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" ht="62" customHeight="1" spans="1:8">
+      <c r="A6" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(m7): complete sprint 3 allocation backlog
</commit_message>
<xml_diff>
--- a/test-evidence/M7-Chai-Zihan/UT-M7-table.xlsx
+++ b/test-evidence/M7-Chai-Zihan/UT-M7-table.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="51">
   <si>
     <t>Test Name/ID</t>
   </si>
@@ -131,19 +131,55 @@
     <t>UT-M7-S3-03</t>
   </si>
   <si>
-    <t>Student already has an accepted application or project has reached capacity</t>
-  </si>
-  <si>
-    <t>Teacher tries to accept another conflicting application</t>
-  </si>
-  <si>
-    <t>System rejects the approval and saves a conflict log</t>
-  </si>
-  <si>
-    <t>System records allocation conflict when student or project capacity conflict occurs</t>
-  </si>
-  <si>
-    <t>Conflict log was saved and approval was rejected</t>
+    <t>Student has other pending applications for different projects</t>
+  </si>
+  <si>
+    <t>Teacher accepts one pending application from this student</t>
+  </si>
+  <si>
+    <t>Other pending applications from the same student are auto rejected and conflict logs are saved</t>
+  </si>
+  <si>
+    <t>Student can only hold one agreed project</t>
+  </si>
+  <si>
+    <t>Other pending applications were rejected after acceptance</t>
+  </si>
+  <si>
+    <t>UT-M7-S3-04</t>
+  </si>
+  <si>
+    <t>Student already has an accepted or agreed project</t>
+  </si>
+  <si>
+    <t>Student tries to submit another application</t>
+  </si>
+  <si>
+    <t>System rejects the application with a conflict message</t>
+  </si>
+  <si>
+    <t>Student cannot apply after already having an agreed project</t>
+  </si>
+  <si>
+    <t>Application was rejected with conflict message</t>
+  </si>
+  <si>
+    <t>UT-M7-S3-05</t>
+  </si>
+  <si>
+    <t>Student has a rejected application and the topic is still available</t>
+  </si>
+  <si>
+    <t>Student submits a new application for the same topic</t>
+  </si>
+  <si>
+    <t>Existing rejected application is updated to pending with new personal statement</t>
+  </si>
+  <si>
+    <t>Student can re-apply after rejection if the topic is available</t>
+  </si>
+  <si>
+    <t>Rejected application became pending and statement was updated</t>
   </si>
 </sst>
 </file>
@@ -323,7 +359,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -333,12 +369,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF2E75B6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.15"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -710,7 +740,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -734,16 +764,16 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -752,85 +782,85 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -851,7 +881,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1200,11 +1230,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="5" outlineLevelCol="7"/>
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="7" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
-    <col min="2" max="2" width="9" customWidth="1"/>
+    <col min="2" max="2" width="12.7272727272727" customWidth="1"/>
     <col min="3" max="3" width="83.6363636363636" customWidth="1"/>
     <col min="4" max="4" width="73.6363636363636" customWidth="1"/>
     <col min="5" max="5" width="70.2727272727273" customWidth="1"/>
@@ -1317,7 +1347,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1" spans="1:8">
+    <row r="5" ht="45" customHeight="1" spans="1:8">
       <c r="A5" s="6" t="s">
         <v>27</v>
       </c>
@@ -1343,7 +1373,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" ht="62" customHeight="1" spans="1:8">
+    <row r="6" ht="43" customHeight="1" spans="1:8">
       <c r="A6" s="6" t="s">
         <v>33</v>
       </c>
@@ -1366,6 +1396,58 @@
         <v>38</v>
       </c>
       <c r="H6" s="6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" ht="39" customHeight="1" spans="1:8">
+      <c r="A7" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" ht="42" spans="1:8">
+      <c r="A8" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="H8" s="6" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>